<commit_message>
chore(data-release): publish site data 2026-10-12 09:43:45 UTC
</commit_message>
<xml_diff>
--- a/countries/br-ac/2026-2029.xlsx
+++ b/countries/br-ac/2026-2029.xlsx
@@ -773,6 +773,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO2" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -909,6 +914,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO3" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -1045,6 +1055,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO4" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -1181,6 +1196,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO5" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -1317,6 +1337,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO6" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -1453,6 +1478,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO7" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -1589,6 +1619,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO8" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -1725,6 +1760,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO9" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -1861,6 +1901,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO10" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -1997,6 +2042,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO11" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -2133,6 +2183,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO12" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -2269,6 +2324,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO13" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -2405,6 +2465,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO14" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -2541,6 +2606,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO15" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -2677,6 +2747,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO16" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -2813,6 +2888,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO17" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -2949,6 +3029,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO18" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -3085,6 +3170,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO19" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -3221,6 +3311,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO20" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -3357,6 +3452,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO21" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -3493,6 +3593,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO22" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -3629,6 +3734,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO23" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -3765,6 +3875,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO24" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -3901,6 +4016,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO25" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -4037,6 +4157,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO26" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -4173,6 +4298,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO27" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -4309,6 +4439,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO28" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -5195,6 +5330,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO33" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -5331,6 +5471,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO34" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -5467,6 +5612,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO35" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -5603,6 +5753,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO36" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -5739,6 +5894,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO37" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -6250,6 +6410,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO40" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -6386,6 +6551,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO41" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -6522,6 +6692,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO42" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -6658,6 +6833,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO43" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -6794,6 +6974,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO44" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -6930,6 +7115,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO45" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -7066,6 +7256,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO46" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -7202,6 +7397,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO47" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -7338,6 +7538,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO48" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -7474,6 +7679,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO49" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -7610,6 +7820,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO50" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -7746,6 +7961,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO51" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -7882,6 +8102,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO52" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -8018,6 +8243,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO53" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -8154,6 +8384,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO54" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -8290,6 +8525,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO55" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -8426,6 +8666,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO56" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -8562,6 +8807,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO57" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -8698,6 +8948,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO58" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -8834,6 +9089,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO59" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -8970,6 +9230,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO60" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -9106,6 +9371,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO61" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -9242,6 +9512,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO62" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -9378,6 +9653,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO63" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -9514,6 +9794,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO64" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -9650,6 +9935,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO65" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -9786,6 +10076,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO66" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -10672,6 +10967,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO71" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -10808,6 +11108,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO72" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -10944,6 +11249,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO73" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -11080,6 +11390,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA74" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO74" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -11591,6 +11906,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA77" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO77" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -12102,6 +12422,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO80" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -12238,6 +12563,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO81" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -12374,6 +12704,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA82" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO82" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -12510,6 +12845,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA83" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO83" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -12782,6 +13122,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA85" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO85" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -12918,6 +13263,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA86" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO86" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -13054,6 +13404,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO87" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -13190,6 +13545,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA88" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO88" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -13326,6 +13686,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA89" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO89" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -13462,6 +13827,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO90" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -13598,6 +13968,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA91" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO91" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -13734,6 +14109,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA92" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO92" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -13870,6 +14250,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA93" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO93" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -14006,6 +14391,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA94" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO94" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -14142,6 +14532,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO95" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -14278,6 +14673,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO96" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -14414,6 +14814,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA97" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO97" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -14550,6 +14955,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA98" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO98" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -14686,6 +15096,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO99" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -14822,6 +15237,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA100" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO100" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -14958,6 +15378,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA101" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO101" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -15094,6 +15519,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA102" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO102" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -15230,6 +15660,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA103" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO103" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -15366,6 +15801,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA104" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO104" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -15502,6 +15942,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA105" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO105" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -16388,6 +16833,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA110" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO110" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -16524,6 +16974,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA111" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO111" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -16660,6 +17115,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA112" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO112" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -17171,6 +17631,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA115" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO115" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -17682,6 +18147,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA118" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO118" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -17818,6 +18288,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA119" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO119" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -17954,6 +18429,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA120" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO120" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -18090,6 +18570,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA121" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO121" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -18226,6 +18711,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA122" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO122" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -18362,6 +18852,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA123" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO123" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -18498,6 +18993,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA124" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO124" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -18634,6 +19134,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA125" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO125" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -18770,6 +19275,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA126" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO126" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -18906,6 +19416,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA127" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO127" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -19042,6 +19557,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA128" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO128" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -19178,6 +19698,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA129" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO129" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -19314,6 +19839,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA130" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO130" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -19450,6 +19980,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA131" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO131" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -19586,6 +20121,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA132" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO132" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -19722,6 +20262,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA133" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO133" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -19858,6 +20403,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA134" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO134" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -19994,6 +20544,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA135" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO135" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -20130,6 +20685,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA136" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO136" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -20266,6 +20826,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA137" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO137" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -20402,6 +20967,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA138" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO138" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -20538,6 +21108,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA139" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO139" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -20674,6 +21249,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA140" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO140" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -20810,6 +21390,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA141" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO141" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -20946,6 +21531,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA142" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO142" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -21082,6 +21672,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA143" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO143" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -21968,6 +22563,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA148" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO148" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -22104,6 +22704,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA149" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO149" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -22240,6 +22845,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA150" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO150" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -22751,6 +23361,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA153" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO153" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -23262,6 +23877,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA156" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO156" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -23398,6 +24018,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA157" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO157" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -23534,6 +24159,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA158" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO158" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -23670,6 +24300,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA159" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO159" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -23806,6 +24441,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA160" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO160" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -23942,6 +24582,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA161" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO161" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -24078,6 +24723,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA162" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO162" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -24214,6 +24864,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA163" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO163" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -24350,6 +25005,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA164" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO164" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -24486,6 +25146,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA165" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO165" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -24622,6 +25287,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA166" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO166" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -24758,6 +25428,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA167" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO167" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -24894,6 +25569,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA168" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO168" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -25030,6 +25710,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA169" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO169" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -25166,6 +25851,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA170" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO170" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -25302,6 +25992,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA171" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO171" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -25438,6 +26133,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA172" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO172" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -25574,6 +26274,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA173" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO173" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -25710,6 +26415,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA174" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO174" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -25846,6 +26556,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA175" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO175" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -25982,6 +26697,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA176" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO176" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -26118,6 +26838,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA177" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO177" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -27004,6 +27729,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA182" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO182" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -27140,6 +27870,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA183" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO183" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -27651,6 +28386,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA186" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO186" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -28162,6 +28902,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA189" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO189" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -28298,6 +29043,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA190" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO190" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -28434,6 +29184,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA191" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO191" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -28570,6 +29325,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA192" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO192" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -28706,6 +29466,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA193" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO193" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -28842,6 +29607,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA194" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO194" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -28978,6 +29748,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA195" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO195" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -29114,6 +29889,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA196" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO196" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -29250,6 +30030,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA197" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO197" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -29386,6 +30171,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA198" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO198" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -29522,6 +30312,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA199" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO199" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -29658,6 +30453,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA200" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO200" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -29794,6 +30594,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA201" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO201" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -29930,6 +30735,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA202" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO202" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -30066,6 +30876,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA203" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO203" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -30202,6 +31017,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA204" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO204" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -30338,6 +31158,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA205" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO205" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -30474,6 +31299,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA206" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO206" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -31360,6 +32190,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA211" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO211" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -31496,6 +32331,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA212" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO212" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -31632,6 +32472,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA213" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO213" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -32143,6 +32988,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA216" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO216" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -32279,6 +33129,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA217" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO217" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -32415,6 +33270,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA218" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO218" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -32551,6 +33411,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA219" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO219" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -32687,6 +33552,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA220" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO220" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -32823,6 +33693,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA221" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO221" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -32959,6 +33834,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA222" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO222" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -33095,6 +33975,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA223" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO223" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -33231,6 +34116,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA224" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO224" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -33367,6 +34257,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA225" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO225" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -33503,6 +34398,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA226" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO226" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -33639,6 +34539,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA227" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO227" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -33775,6 +34680,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA228" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO228" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -33911,6 +34821,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA229" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO229" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -34047,6 +34962,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA230" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO230" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -34183,6 +35103,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA231" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO231" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -34319,6 +35244,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA232" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO232" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -35205,6 +36135,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA237" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO237" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -35341,6 +36276,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA238" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO238" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -35477,6 +36417,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA239" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO239" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -35988,6 +36933,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA242" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO242" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -36124,6 +37074,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA243" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO243" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -36260,6 +37215,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA244" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO244" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -36396,6 +37356,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA245" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO245" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -36532,6 +37497,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA246" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO246" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -36668,6 +37638,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA247" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO247" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -36804,6 +37779,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA248" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO248" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -36940,6 +37920,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA249" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO249" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -37076,6 +38061,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA250" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO250" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -37212,6 +38202,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA251" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO251" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -37348,6 +38343,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA252" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO252" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -37484,6 +38484,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA253" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO253" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -37620,6 +38625,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA254" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO254" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -37756,6 +38766,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA255" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO255" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -37892,6 +38907,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA256" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO256" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -38778,6 +39798,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA261" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO261" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -38914,6 +39939,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA262" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO262" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -39050,6 +40080,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA263" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO263" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -39561,6 +40596,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA266" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO266" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -39697,6 +40737,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA267" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO267" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -39833,6 +40878,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA268" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO268" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -39969,6 +41019,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA269" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO269" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -40105,6 +41160,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA270" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO270" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -40241,6 +41301,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA271" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO271" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -40377,6 +41442,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA272" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO272" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -40513,6 +41583,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA273" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO273" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -40649,6 +41724,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA274" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO274" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -40785,6 +41865,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA275" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO275" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -40921,6 +42006,11 @@
           <t>ibge_computed</t>
         </is>
       </c>
+      <c r="AA276" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO276" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
@@ -41055,6 +42145,11 @@
       <c r="S277" t="inlineStr">
         <is>
           <t>ibge_computed</t>
+        </is>
+      </c>
+      <c r="AA277" t="inlineStr">
+        <is>
+          <t>monthly</t>
         </is>
       </c>
       <c r="AO277" t="inlineStr">

</xml_diff>